<commit_message>
Schematic ready for review
</commit_message>
<xml_diff>
--- a/Simulations/Temperature vs Voltage.xlsx
+++ b/Simulations/Temperature vs Voltage.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dylan\Documents\GitHub\Black_Body\simulation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dylan\Documents\GitHub\Black_Body\Simulations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB89547B-CBF1-413D-ADA8-AECEFF11AC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08BF9C9-DEAF-4B36-8603-CF8CE70FA52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="218" yWindow="900" windowWidth="21164" windowHeight="11662" xr2:uid="{6FDD085B-2125-46E3-9E49-998CCF20B50B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{6FDD085B-2125-46E3-9E49-998CCF20B50B}"/>
   </bookViews>
   <sheets>
     <sheet name="Graph" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>Temperature (k)</t>
   </si>
@@ -71,6 +71,9 @@
   <si>
     <t>&lt;0.1mV</t>
   </si>
+  <si>
+    <t>0.01uA</t>
+  </si>
 </sst>
 </file>
 
@@ -78,7 +81,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -135,23 +138,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -275,7 +274,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.1uA</c:v>
+                  <c:v>0.01uA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -304,42 +303,6 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:cat>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="10"/>
-              <c:pt idx="0">
-                <c:v>0.3</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>0.5</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>1</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>1.4</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>2</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>4.2</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="7">
-                <c:v>40</c:v>
-              </c:pt>
-              <c:pt idx="8">
-                <c:v>77.400000000000006</c:v>
-              </c:pt>
-              <c:pt idx="9">
-                <c:v>100</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Graph!$B$3:$B$12</c:f>
@@ -347,34 +310,34 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>3.5179999999999998</c:v>
+                  <c:v>0.3518</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5442999999999999</c:v>
+                  <c:v>5.4429999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.7570000000000009E-2</c:v>
+                  <c:v>8.7570000000000009E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.4860000000000004E-2</c:v>
+                  <c:v>4.4859999999999995E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4879999999999999E-2</c:v>
+                  <c:v>2.4880000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9.4459999999999995E-3</c:v>
+                  <c:v>9.4459999999999998E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.32E-3</c:v>
+                  <c:v>3.3200000000000005E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.7890000000000001E-4</c:v>
+                  <c:v>7.7890000000000001E-5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.5039999999999995E-4</c:v>
+                  <c:v>3.5040000000000003E-5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.7160000000000004E-4</c:v>
+                  <c:v>2.7160000000000004E-5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -395,7 +358,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1uA</c:v>
+                  <c:v>0.1uA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -424,42 +387,6 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:cat>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="10"/>
-              <c:pt idx="0">
-                <c:v>0.3</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>0.5</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>1</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>1.4</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>2</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>4.2</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="7">
-                <c:v>40</c:v>
-              </c:pt>
-              <c:pt idx="8">
-                <c:v>77.400000000000006</c:v>
-              </c:pt>
-              <c:pt idx="9">
-                <c:v>100</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Graph!$C$3:$C$12</c:f>
@@ -467,34 +394,34 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>35.179999999999993</c:v>
+                  <c:v>3.5179999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.4429999999999996</c:v>
+                  <c:v>0.5442999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.87570000000000003</c:v>
+                  <c:v>8.7570000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4486</c:v>
+                  <c:v>4.4860000000000004E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.24879999999999997</c:v>
+                  <c:v>2.4879999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9.4459999999999988E-2</c:v>
+                  <c:v>9.4459999999999995E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.32E-2</c:v>
+                  <c:v>3.32E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.788999999999999E-3</c:v>
+                  <c:v>7.7890000000000001E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.5039999999999997E-3</c:v>
+                  <c:v>3.5039999999999995E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.7160000000000001E-3</c:v>
+                  <c:v>2.7160000000000004E-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -515,7 +442,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>10uA</c:v>
+                  <c:v>1uA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -544,42 +471,6 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:cat>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="10"/>
-              <c:pt idx="0">
-                <c:v>0.3</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>0.5</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>1</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>1.4</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>2</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>4.2</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="7">
-                <c:v>40</c:v>
-              </c:pt>
-              <c:pt idx="8">
-                <c:v>77.400000000000006</c:v>
-              </c:pt>
-              <c:pt idx="9">
-                <c:v>100</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Graph!$D$3:$D$12</c:f>
@@ -587,34 +478,34 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>351.79999999999995</c:v>
+                  <c:v>35.179999999999993</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>54.429999999999993</c:v>
+                  <c:v>5.4429999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.7569999999999997</c:v>
+                  <c:v>0.87570000000000003</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.4859999999999998</c:v>
+                  <c:v>0.4486</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4879999999999995</c:v>
+                  <c:v>0.24879999999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.94459999999999988</c:v>
+                  <c:v>9.4459999999999988E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.33200000000000002</c:v>
+                  <c:v>3.32E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.7889999999999987E-2</c:v>
+                  <c:v>7.788999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.5039999999999995E-2</c:v>
+                  <c:v>3.5039999999999997E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.716E-2</c:v>
+                  <c:v>2.7160000000000001E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -635,7 +526,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>100uA</c:v>
+                  <c:v>10uA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -658,48 +549,12 @@
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent1"/>
+                  <a:schemeClr val="accent4"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:cat>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="10"/>
-              <c:pt idx="0">
-                <c:v>0.3</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>0.5</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>1</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>1.4</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>2</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>4.2</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="7">
-                <c:v>40</c:v>
-              </c:pt>
-              <c:pt idx="8">
-                <c:v>77.400000000000006</c:v>
-              </c:pt>
-              <c:pt idx="9">
-                <c:v>100</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Graph!$E$3:$E$12</c:f>
@@ -707,34 +562,34 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>3518</c:v>
+                  <c:v>351.79999999999995</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>544.29999999999995</c:v>
+                  <c:v>54.429999999999993</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>87.57</c:v>
+                  <c:v>8.7569999999999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>44.86</c:v>
+                  <c:v>4.4859999999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24.88</c:v>
+                  <c:v>2.4879999999999995</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9.445999999999998</c:v>
+                  <c:v>0.94459999999999988</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.32</c:v>
+                  <c:v>0.33200000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.77889999999999993</c:v>
+                  <c:v>7.7889999999999987E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.35039999999999993</c:v>
+                  <c:v>3.5039999999999995E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.27160000000000001</c:v>
+                  <c:v>2.716E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -755,7 +610,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>1000uA</c:v>
+                  <c:v>100uA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -778,48 +633,12 @@
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent5"/>
+                  <a:schemeClr val="accent1"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:cat>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="10"/>
-              <c:pt idx="0">
-                <c:v>0.3</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>0.5</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>1</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>1.4</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>2</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>4.2</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>10</c:v>
-              </c:pt>
-              <c:pt idx="7">
-                <c:v>40</c:v>
-              </c:pt>
-              <c:pt idx="8">
-                <c:v>77.400000000000006</c:v>
-              </c:pt>
-              <c:pt idx="9">
-                <c:v>100</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Graph!$F$3:$F$12</c:f>
@@ -827,34 +646,34 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>35180</c:v>
+                  <c:v>3518</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5443.0000000000009</c:v>
+                  <c:v>544.29999999999995</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>875.7</c:v>
+                  <c:v>87.57</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>448.60000000000008</c:v>
+                  <c:v>44.86</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>248.8</c:v>
+                  <c:v>24.88</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>94.460000000000008</c:v>
+                  <c:v>9.445999999999998</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>33.200000000000003</c:v>
+                  <c:v>3.32</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.7889999999999997</c:v>
+                  <c:v>0.77889999999999993</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.504</c:v>
+                  <c:v>0.35039999999999993</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.7160000000000002</c:v>
+                  <c:v>0.27160000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -863,6 +682,90 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-E8E8-4879-A91B-C7CD65F8E213}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Graph!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1000uA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Graph!$G$3:$G$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>35180</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5443.0000000000009</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>875.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>448.60000000000008</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>248.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>94.460000000000008</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>33.200000000000003</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.7889999999999997</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.504</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.7160000000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-49D2-4B90-8D4A-5428E8AEBC10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1742,13 +1645,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>531018</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>28574</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>61232</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>176892</xdr:rowOff>
@@ -2096,301 +1999,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A2D628-D98E-4197-8325-6E39B43513B2}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.6640625" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>35180</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <f>Data!C3</f>
+        <v>0.3518</v>
+      </c>
+      <c r="C3" s="4">
+        <f>Data!D3</f>
         <v>3.5179999999999998</v>
       </c>
-      <c r="C3" s="6">
-        <f>Data!D3</f>
+      <c r="D3" s="4">
+        <f>Data!E3</f>
         <v>35.179999999999993</v>
       </c>
-      <c r="D3" s="6">
-        <f>Data!E3</f>
+      <c r="E3" s="4">
+        <f>Data!F3</f>
         <v>351.79999999999995</v>
       </c>
-      <c r="E3" s="6">
-        <f>Data!F3</f>
+      <c r="F3" s="4">
+        <f>Data!G3</f>
         <v>3518</v>
       </c>
-      <c r="F3" s="6">
-        <f>Data!G3</f>
+      <c r="G3" s="4">
+        <f>Data!H3</f>
         <v>35180</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>5443</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <f>Data!C4</f>
+        <v>5.4429999999999999E-2</v>
+      </c>
+      <c r="C4" s="4">
+        <f>Data!D4</f>
         <v>0.5442999999999999</v>
       </c>
-      <c r="C4" s="6">
-        <f>Data!D4</f>
+      <c r="D4" s="4">
+        <f>Data!E4</f>
         <v>5.4429999999999996</v>
       </c>
-      <c r="D4" s="6">
-        <f>Data!E4</f>
+      <c r="E4" s="4">
+        <f>Data!F4</f>
         <v>54.429999999999993</v>
       </c>
-      <c r="E4" s="6">
-        <f>Data!F4</f>
+      <c r="F4" s="4">
+        <f>Data!G4</f>
         <v>544.29999999999995</v>
       </c>
-      <c r="F4" s="6">
-        <f>Data!G4</f>
+      <c r="G4" s="4">
+        <f>Data!H4</f>
         <v>5443.0000000000009</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>875.7</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <f>Data!C5</f>
+        <v>8.7570000000000009E-3</v>
+      </c>
+      <c r="C5" s="4">
+        <f>Data!D5</f>
         <v>8.7570000000000009E-2</v>
       </c>
-      <c r="C5" s="6">
-        <f>Data!D5</f>
+      <c r="D5" s="4">
+        <f>Data!E5</f>
         <v>0.87570000000000003</v>
       </c>
-      <c r="D5" s="6">
-        <f>Data!E5</f>
+      <c r="E5" s="4">
+        <f>Data!F5</f>
         <v>8.7569999999999997</v>
       </c>
-      <c r="E5" s="6">
-        <f>Data!F5</f>
+      <c r="F5" s="4">
+        <f>Data!G5</f>
         <v>87.57</v>
       </c>
-      <c r="F5" s="6">
-        <f>Data!G5</f>
+      <c r="G5" s="4">
+        <f>Data!H5</f>
         <v>875.7</v>
       </c>
-      <c r="I5" s="13"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>448.6</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <f>Data!C6</f>
+        <v>4.4859999999999995E-3</v>
+      </c>
+      <c r="C6" s="4">
+        <f>Data!D6</f>
         <v>4.4860000000000004E-2</v>
       </c>
-      <c r="C6" s="6">
-        <f>Data!D6</f>
+      <c r="D6" s="4">
+        <f>Data!E6</f>
         <v>0.4486</v>
       </c>
-      <c r="D6" s="6">
-        <f>Data!E6</f>
+      <c r="E6" s="4">
+        <f>Data!F6</f>
         <v>4.4859999999999998</v>
       </c>
-      <c r="E6" s="6">
-        <f>Data!F6</f>
+      <c r="F6" s="4">
+        <f>Data!G6</f>
         <v>44.86</v>
       </c>
-      <c r="F6" s="6">
-        <f>Data!G6</f>
+      <c r="G6" s="4">
+        <f>Data!H6</f>
         <v>448.60000000000008</v>
       </c>
-      <c r="I6" s="13"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>248.8</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <f>Data!C7</f>
+        <v>2.4880000000000002E-3</v>
+      </c>
+      <c r="C7" s="4">
+        <f>Data!D7</f>
         <v>2.4879999999999999E-2</v>
       </c>
-      <c r="C7" s="6">
-        <f>Data!D7</f>
+      <c r="D7" s="4">
+        <f>Data!E7</f>
         <v>0.24879999999999997</v>
       </c>
-      <c r="D7" s="6">
-        <f>Data!E7</f>
+      <c r="E7" s="4">
+        <f>Data!F7</f>
         <v>2.4879999999999995</v>
       </c>
-      <c r="E7" s="6">
-        <f>Data!F7</f>
+      <c r="F7" s="4">
+        <f>Data!G7</f>
         <v>24.88</v>
       </c>
-      <c r="F7" s="6">
-        <f>Data!G7</f>
+      <c r="G7" s="4">
+        <f>Data!H7</f>
         <v>248.8</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>94.46</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="4">
         <f>Data!C8</f>
+        <v>9.4459999999999998E-4</v>
+      </c>
+      <c r="C8" s="4">
+        <f>Data!D8</f>
         <v>9.4459999999999995E-3</v>
       </c>
-      <c r="C8" s="6">
-        <f>Data!D8</f>
+      <c r="D8" s="4">
+        <f>Data!E8</f>
         <v>9.4459999999999988E-2</v>
       </c>
-      <c r="D8" s="6">
-        <f>Data!E8</f>
+      <c r="E8" s="4">
+        <f>Data!F8</f>
         <v>0.94459999999999988</v>
       </c>
-      <c r="E8" s="6">
-        <f>Data!F8</f>
+      <c r="F8" s="4">
+        <f>Data!G8</f>
         <v>9.445999999999998</v>
       </c>
-      <c r="F8" s="6">
-        <f>Data!G8</f>
+      <c r="G8" s="4">
+        <f>Data!H8</f>
         <v>94.460000000000008</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>33.200000000000003</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>Data!C9</f>
+        <v>3.3200000000000005E-4</v>
+      </c>
+      <c r="C9" s="4">
+        <f>Data!D9</f>
         <v>3.32E-3</v>
       </c>
-      <c r="C9" s="6">
-        <f>Data!D9</f>
+      <c r="D9" s="4">
+        <f>Data!E9</f>
         <v>3.32E-2</v>
       </c>
-      <c r="D9" s="6">
-        <f>Data!E9</f>
+      <c r="E9" s="4">
+        <f>Data!F9</f>
         <v>0.33200000000000002</v>
       </c>
-      <c r="E9" s="6">
-        <f>Data!F9</f>
+      <c r="F9" s="4">
+        <f>Data!G9</f>
         <v>3.32</v>
       </c>
-      <c r="F9" s="6">
-        <f>Data!G9</f>
+      <c r="G9" s="4">
+        <f>Data!H9</f>
         <v>33.200000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>7.7889999999999997</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="4">
         <f>Data!C10</f>
+        <v>7.7890000000000001E-5</v>
+      </c>
+      <c r="C10" s="4">
+        <f>Data!D10</f>
         <v>7.7890000000000001E-4</v>
       </c>
-      <c r="C10" s="6">
-        <f>Data!D10</f>
+      <c r="D10" s="4">
+        <f>Data!E10</f>
         <v>7.788999999999999E-3</v>
       </c>
-      <c r="D10" s="6">
-        <f>Data!E10</f>
+      <c r="E10" s="4">
+        <f>Data!F10</f>
         <v>7.7889999999999987E-2</v>
       </c>
-      <c r="E10" s="6">
-        <f>Data!F10</f>
+      <c r="F10" s="4">
+        <f>Data!G10</f>
         <v>0.77889999999999993</v>
       </c>
-      <c r="F10" s="6">
-        <f>Data!G10</f>
+      <c r="G10" s="4">
+        <f>Data!H10</f>
         <v>7.7889999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>3.504</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="4">
         <f>Data!C11</f>
+        <v>3.5040000000000003E-5</v>
+      </c>
+      <c r="C11" s="4">
+        <f>Data!D11</f>
         <v>3.5039999999999995E-4</v>
       </c>
-      <c r="C11" s="6">
-        <f>Data!D11</f>
+      <c r="D11" s="4">
+        <f>Data!E11</f>
         <v>3.5039999999999997E-3</v>
       </c>
-      <c r="D11" s="6">
-        <f>Data!E11</f>
+      <c r="E11" s="4">
+        <f>Data!F11</f>
         <v>3.5039999999999995E-2</v>
       </c>
-      <c r="E11" s="6">
-        <f>Data!F11</f>
+      <c r="F11" s="4">
+        <f>Data!G11</f>
         <v>0.35039999999999993</v>
       </c>
-      <c r="F11" s="6">
-        <f>Data!G11</f>
+      <c r="G11" s="4">
+        <f>Data!H11</f>
         <v>3.504</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2.7160000000000002</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="4">
         <f>Data!C12</f>
+        <v>2.7160000000000004E-5</v>
+      </c>
+      <c r="C12" s="4">
+        <f>Data!D12</f>
         <v>2.7160000000000004E-4</v>
       </c>
-      <c r="C12" s="6">
-        <f>Data!D12</f>
+      <c r="D12" s="4">
+        <f>Data!E12</f>
         <v>2.7160000000000001E-3</v>
       </c>
-      <c r="D12" s="6">
-        <f>Data!E12</f>
+      <c r="E12" s="4">
+        <f>Data!F12</f>
         <v>2.716E-2</v>
       </c>
-      <c r="E12" s="6">
-        <f>Data!F12</f>
+      <c r="F12" s="4">
+        <f>Data!G12</f>
         <v>0.27160000000000001</v>
       </c>
-      <c r="F12" s="6">
-        <f>Data!G12</f>
+      <c r="G12" s="4">
+        <f>Data!H12</f>
         <v>2.7160000000000002</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2399,340 +2345,385 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E40DC60C-1FCE-4293-9A3D-709A089882DB}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="4" max="4" width="9.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="C1" s="3" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="D1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
+        <f>0.01*10^-6</f>
+        <v>1E-8</v>
+      </c>
+      <c r="D2" s="3">
         <f>0.1*10^-6</f>
         <v>9.9999999999999995E-8</v>
       </c>
-      <c r="D2" s="4">
+      <c r="E2" s="3">
         <f>1*10^-6</f>
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F2" s="3">
         <f>10*10^-6</f>
         <v>9.9999999999999991E-6</v>
       </c>
-      <c r="F2" s="4">
+      <c r="G2" s="3">
         <f>100*10^-6</f>
         <v>9.9999999999999991E-5</v>
       </c>
-      <c r="G2" s="4">
+      <c r="H2" s="3">
         <f>1000*10^-6</f>
         <v>1E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>0.3</v>
       </c>
       <c r="B3">
         <v>35180</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="4">
         <f>$C$2*B3*1000</f>
+        <v>0.3518</v>
+      </c>
+      <c r="D3" s="4">
+        <f>$D$2*B3*1000</f>
         <v>3.5179999999999998</v>
       </c>
-      <c r="D3" s="7">
-        <f>$D$2*B3*1000</f>
+      <c r="E3" s="5">
+        <f>$E$2*B3*1000</f>
         <v>35.179999999999993</v>
       </c>
-      <c r="E3" s="7">
-        <f>$E$2*B3*1000</f>
+      <c r="F3" s="5">
+        <f>$F$2*B3*1000</f>
         <v>351.79999999999995</v>
       </c>
-      <c r="F3" s="7">
-        <f>$F$2*B3*1000</f>
+      <c r="G3" s="5">
+        <f>$G$2*B3*1000</f>
         <v>3518</v>
       </c>
-      <c r="G3" s="7">
-        <f>$G$2*B3*1000</f>
+      <c r="H3" s="5">
+        <f>$H$2*B3*1000</f>
         <v>35180</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>0.5</v>
       </c>
       <c r="B4">
         <v>5443</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="8">
         <f t="shared" ref="C4:C12" si="0">$C$2*B4*1000</f>
+        <v>5.4429999999999999E-2</v>
+      </c>
+      <c r="D4" s="4">
+        <f t="shared" ref="D4:D12" si="1">$D$2*B4*1000</f>
         <v>0.5442999999999999</v>
       </c>
-      <c r="D4" s="5">
-        <f t="shared" ref="D4:D12" si="1">$D$2*B4*1000</f>
+      <c r="E4">
+        <f t="shared" ref="E4:E12" si="2">$E$2*B4*1000</f>
         <v>5.4429999999999996</v>
       </c>
-      <c r="E4" s="8">
-        <f t="shared" ref="E4:E12" si="2">$E$2*B4*1000</f>
+      <c r="F4" s="6">
+        <f t="shared" ref="F4:F12" si="3">$F$2*B4*1000</f>
         <v>54.429999999999993</v>
       </c>
-      <c r="F4" s="8">
-        <f t="shared" ref="F4:F12" si="3">$F$2*B4*1000</f>
+      <c r="G4" s="6">
+        <f t="shared" ref="G4:G12" si="4">$G$2*B4*1000</f>
         <v>544.29999999999995</v>
       </c>
-      <c r="G4" s="8">
-        <f t="shared" ref="G4:G12" si="4">$G$2*B4*1000</f>
+      <c r="H4" s="6">
+        <f t="shared" ref="H4:H12" si="5">$H$2*B4*1000</f>
         <v>5443.0000000000009</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>1</v>
       </c>
       <c r="B5">
         <v>875.7</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="8">
         <f t="shared" si="0"/>
+        <v>8.7570000000000009E-3</v>
+      </c>
+      <c r="D5" s="8">
+        <f t="shared" si="1"/>
         <v>8.7570000000000009E-2</v>
       </c>
-      <c r="D5" s="5">
-        <f t="shared" si="1"/>
+      <c r="E5">
+        <f t="shared" si="2"/>
         <v>0.87570000000000003</v>
       </c>
-      <c r="E5" s="5">
-        <f t="shared" si="2"/>
+      <c r="F5">
+        <f t="shared" si="3"/>
         <v>8.7569999999999997</v>
       </c>
-      <c r="F5" s="8">
-        <f t="shared" si="3"/>
+      <c r="G5" s="6">
+        <f t="shared" si="4"/>
         <v>87.57</v>
       </c>
-      <c r="G5" s="8">
-        <f t="shared" si="4"/>
+      <c r="H5" s="6">
+        <f t="shared" si="5"/>
         <v>875.7</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>1.4</v>
       </c>
       <c r="B6">
         <v>448.6</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="8">
         <f t="shared" si="0"/>
+        <v>4.4859999999999995E-3</v>
+      </c>
+      <c r="D6" s="8">
+        <f t="shared" si="1"/>
         <v>4.4860000000000004E-2</v>
       </c>
-      <c r="D6" s="5">
-        <f t="shared" si="1"/>
+      <c r="E6">
+        <f t="shared" si="2"/>
         <v>0.4486</v>
       </c>
-      <c r="E6" s="5">
-        <f t="shared" si="2"/>
+      <c r="F6">
+        <f t="shared" si="3"/>
         <v>4.4859999999999998</v>
       </c>
-      <c r="F6" s="8">
-        <f t="shared" si="3"/>
+      <c r="G6" s="6">
+        <f t="shared" si="4"/>
         <v>44.86</v>
       </c>
-      <c r="G6" s="8">
-        <f t="shared" si="4"/>
+      <c r="H6" s="6">
+        <f t="shared" si="5"/>
         <v>448.60000000000008</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="K6" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>2</v>
       </c>
       <c r="B7">
         <v>248.8</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="8">
         <f t="shared" si="0"/>
+        <v>2.4880000000000002E-3</v>
+      </c>
+      <c r="D7" s="8">
+        <f t="shared" si="1"/>
         <v>2.4879999999999999E-2</v>
       </c>
-      <c r="D7" s="5">
-        <f t="shared" si="1"/>
+      <c r="E7">
+        <f t="shared" si="2"/>
         <v>0.24879999999999997</v>
       </c>
-      <c r="E7" s="5">
-        <f t="shared" si="2"/>
+      <c r="F7">
+        <f t="shared" si="3"/>
         <v>2.4879999999999995</v>
       </c>
-      <c r="F7" s="8">
-        <f t="shared" si="3"/>
+      <c r="G7" s="6">
+        <f t="shared" si="4"/>
         <v>24.88</v>
       </c>
-      <c r="G7" s="8">
-        <f t="shared" si="4"/>
+      <c r="H7" s="6">
+        <f t="shared" si="5"/>
         <v>248.8</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>4.2</v>
       </c>
       <c r="B8">
         <v>94.46</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="8">
         <f t="shared" si="0"/>
+        <v>9.4459999999999998E-4</v>
+      </c>
+      <c r="D8" s="8">
+        <f t="shared" si="1"/>
         <v>9.4459999999999995E-3</v>
       </c>
-      <c r="D8" s="12">
-        <f t="shared" si="1"/>
+      <c r="E8" s="7">
+        <f t="shared" si="2"/>
         <v>9.4459999999999988E-2</v>
       </c>
-      <c r="E8" s="5">
-        <f t="shared" si="2"/>
+      <c r="F8">
+        <f t="shared" si="3"/>
         <v>0.94459999999999988</v>
       </c>
-      <c r="F8" s="5">
-        <f t="shared" si="3"/>
+      <c r="G8">
+        <f t="shared" si="4"/>
         <v>9.445999999999998</v>
       </c>
-      <c r="G8" s="8">
-        <f t="shared" si="4"/>
+      <c r="H8" s="6">
+        <f t="shared" si="5"/>
         <v>94.460000000000008</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>10</v>
       </c>
       <c r="B9">
         <v>33.200000000000003</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="8">
         <f t="shared" si="0"/>
+        <v>3.3200000000000005E-4</v>
+      </c>
+      <c r="D9" s="8">
+        <f t="shared" si="1"/>
         <v>3.32E-3</v>
       </c>
-      <c r="D9" s="12">
-        <f t="shared" si="1"/>
+      <c r="E9" s="7">
+        <f t="shared" si="2"/>
         <v>3.32E-2</v>
       </c>
-      <c r="E9" s="5">
-        <f t="shared" si="2"/>
+      <c r="F9">
+        <f t="shared" si="3"/>
         <v>0.33200000000000002</v>
       </c>
-      <c r="F9" s="5">
-        <f t="shared" si="3"/>
+      <c r="G9">
+        <f t="shared" si="4"/>
         <v>3.32</v>
       </c>
-      <c r="G9" s="8">
-        <f t="shared" si="4"/>
+      <c r="H9" s="6">
+        <f t="shared" si="5"/>
         <v>33.200000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>40</v>
       </c>
       <c r="B10">
         <v>7.7889999999999997</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="8">
         <f t="shared" si="0"/>
+        <v>7.7890000000000001E-5</v>
+      </c>
+      <c r="D10" s="8">
+        <f t="shared" si="1"/>
         <v>7.7890000000000001E-4</v>
       </c>
-      <c r="D10" s="12">
-        <f t="shared" si="1"/>
+      <c r="E10" s="7">
+        <f t="shared" si="2"/>
         <v>7.788999999999999E-3</v>
       </c>
-      <c r="E10" s="12">
-        <f t="shared" si="2"/>
+      <c r="F10" s="7">
+        <f t="shared" si="3"/>
         <v>7.7889999999999987E-2</v>
       </c>
-      <c r="F10" s="5">
-        <f t="shared" si="3"/>
+      <c r="G10">
+        <f t="shared" si="4"/>
         <v>0.77889999999999993</v>
       </c>
-      <c r="G10" s="5">
-        <f t="shared" si="4"/>
+      <c r="H10">
+        <f t="shared" si="5"/>
         <v>7.7889999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>77.400000000000006</v>
       </c>
       <c r="B11">
         <v>3.504</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="8">
         <f t="shared" si="0"/>
+        <v>3.5040000000000003E-5</v>
+      </c>
+      <c r="D11" s="8">
+        <f t="shared" si="1"/>
         <v>3.5039999999999995E-4</v>
       </c>
-      <c r="D11" s="12">
-        <f t="shared" si="1"/>
+      <c r="E11" s="7">
+        <f t="shared" si="2"/>
         <v>3.5039999999999997E-3</v>
       </c>
-      <c r="E11" s="12">
-        <f t="shared" si="2"/>
+      <c r="F11" s="7">
+        <f t="shared" si="3"/>
         <v>3.5039999999999995E-2</v>
       </c>
-      <c r="F11" s="5">
-        <f t="shared" si="3"/>
+      <c r="G11">
+        <f t="shared" si="4"/>
         <v>0.35039999999999993</v>
       </c>
-      <c r="G11" s="5">
-        <f t="shared" si="4"/>
+      <c r="H11">
+        <f t="shared" si="5"/>
         <v>3.504</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>100</v>
       </c>
       <c r="B12">
         <v>2.7160000000000002</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="8">
         <f t="shared" si="0"/>
+        <v>2.7160000000000004E-5</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" si="1"/>
         <v>2.7160000000000004E-4</v>
       </c>
-      <c r="D12" s="12">
-        <f t="shared" si="1"/>
+      <c r="E12" s="7">
+        <f t="shared" si="2"/>
         <v>2.7160000000000001E-3</v>
       </c>
-      <c r="E12" s="12">
-        <f t="shared" si="2"/>
+      <c r="F12" s="7">
+        <f t="shared" si="3"/>
         <v>2.716E-2</v>
       </c>
-      <c r="F12" s="5">
-        <f t="shared" si="3"/>
+      <c r="G12">
+        <f t="shared" si="4"/>
         <v>0.27160000000000001</v>
       </c>
-      <c r="G12" s="5">
-        <f t="shared" si="4"/>
+      <c r="H12">
+        <f t="shared" si="5"/>
         <v>2.7160000000000002</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="D1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>